<commit_message>
completed data dictionary and query quality log from sql profiling
</commit_message>
<xml_diff>
--- a/Data_Dictionary_IPL_Completed.xlsx
+++ b/Data_Dictionary_IPL_Completed.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muhju\Downloads\test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/378e640fabecb426/Desktop/ipl. project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A40C5B-45F7-4464-BCF2-2A84F210D85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{E7A40C5B-45F7-4464-BCF2-2A84F210D85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B25F9CA7-2D12-426C-B1E0-D8653F96A76E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2. Relationships'!$A$4:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'3. Data Quality Log'!$A$4:$F$35</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -33,8 +33,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -1727,9 +1725,6 @@
     <t>IPL CRICKET ANALYTICS</t>
   </si>
   <si>
-    <t>Muhammed Junaid pk</t>
-  </si>
-  <si>
     <t>Company-provided SQLite database (ipl.db)</t>
   </si>
   <si>
@@ -1740,6 +1735,9 @@
   </si>
   <si>
     <t>44.77mb</t>
+  </si>
+  <si>
+    <t>ayas nk</t>
   </si>
 </sst>
 </file>
@@ -2029,20 +2027,6 @@
     <xf numFmtId="0" fontId="11" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2052,6 +2036,20 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2522,14 +2520,14 @@
         <v>51</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="37">
+      <c r="C7" s="29">
         <v>46251</v>
       </c>
     </row>
@@ -2538,7 +2536,7 @@
         <v>53</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2546,22 +2544,22 @@
         <v>54</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="38" t="s">
-        <v>562</v>
+      <c r="C10" s="30" t="s">
+        <v>561</v>
       </c>
     </row>
     <row r="11" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="39">
+      <c r="C11" s="31">
         <v>5</v>
       </c>
     </row>
@@ -2569,8 +2567,8 @@
       <c r="B12" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C12" s="38" t="s">
-        <v>563</v>
+      <c r="C12" s="30" t="s">
+        <v>562</v>
       </c>
     </row>
   </sheetData>
@@ -2593,132 +2591,132 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="30"/>
-      <c r="T1" s="30"/>
-      <c r="U1" s="30"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
+      <c r="O1" s="33"/>
+      <c r="P1" s="33"/>
+      <c r="Q1" s="33"/>
+      <c r="R1" s="33"/>
+      <c r="S1" s="33"/>
+      <c r="T1" s="33"/>
+      <c r="U1" s="33"/>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="39" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="30"/>
-      <c r="P2" s="30"/>
-      <c r="Q2" s="30"/>
-      <c r="R2" s="30"/>
-      <c r="S2" s="30"/>
-      <c r="T2" s="30"/>
-      <c r="U2" s="30"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="33"/>
+      <c r="O2" s="33"/>
+      <c r="P2" s="33"/>
+      <c r="Q2" s="33"/>
+      <c r="R2" s="33"/>
+      <c r="S2" s="33"/>
+      <c r="T2" s="33"/>
+      <c r="U2" s="33"/>
     </row>
     <row r="4" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="33"/>
-      <c r="J4" s="33"/>
-      <c r="K4" s="33"/>
-      <c r="L4" s="33"/>
-      <c r="M4" s="33"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="33"/>
-      <c r="P4" s="33"/>
-      <c r="Q4" s="33"/>
-      <c r="R4" s="33"/>
-      <c r="S4" s="33"/>
-      <c r="T4" s="33"/>
-      <c r="U4" s="33"/>
-      <c r="V4" s="33"/>
-      <c r="W4" s="33"/>
-      <c r="X4" s="33"/>
-      <c r="Y4" s="33"/>
-      <c r="Z4" s="33"/>
-      <c r="AA4" s="33"/>
-      <c r="AB4" s="33"/>
-      <c r="AC4" s="33"/>
-      <c r="AD4" s="33"/>
-      <c r="AE4" s="33"/>
-      <c r="AF4" s="33"/>
-      <c r="AG4" s="34"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
+      <c r="K4" s="35"/>
+      <c r="L4" s="35"/>
+      <c r="M4" s="35"/>
+      <c r="N4" s="35"/>
+      <c r="O4" s="35"/>
+      <c r="P4" s="35"/>
+      <c r="Q4" s="35"/>
+      <c r="R4" s="35"/>
+      <c r="S4" s="35"/>
+      <c r="T4" s="35"/>
+      <c r="U4" s="35"/>
+      <c r="V4" s="35"/>
+      <c r="W4" s="35"/>
+      <c r="X4" s="35"/>
+      <c r="Y4" s="35"/>
+      <c r="Z4" s="35"/>
+      <c r="AA4" s="35"/>
+      <c r="AB4" s="35"/>
+      <c r="AC4" s="35"/>
+      <c r="AD4" s="35"/>
+      <c r="AE4" s="35"/>
+      <c r="AF4" s="35"/>
+      <c r="AG4" s="36"/>
     </row>
     <row r="5" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="37" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="33"/>
-      <c r="I5" s="33"/>
-      <c r="J5" s="33"/>
-      <c r="K5" s="33"/>
-      <c r="L5" s="33"/>
-      <c r="M5" s="33"/>
-      <c r="N5" s="33"/>
-      <c r="O5" s="33"/>
-      <c r="P5" s="33"/>
-      <c r="Q5" s="33"/>
-      <c r="R5" s="33"/>
-      <c r="S5" s="33"/>
-      <c r="T5" s="33"/>
-      <c r="U5" s="33"/>
-      <c r="V5" s="33"/>
-      <c r="W5" s="33"/>
-      <c r="X5" s="33"/>
-      <c r="Y5" s="33"/>
-      <c r="Z5" s="33"/>
-      <c r="AA5" s="33"/>
-      <c r="AB5" s="33"/>
-      <c r="AC5" s="33"/>
-      <c r="AD5" s="33"/>
-      <c r="AE5" s="33"/>
-      <c r="AF5" s="33"/>
-      <c r="AG5" s="34"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="35"/>
+      <c r="J5" s="35"/>
+      <c r="K5" s="35"/>
+      <c r="L5" s="35"/>
+      <c r="M5" s="35"/>
+      <c r="N5" s="35"/>
+      <c r="O5" s="35"/>
+      <c r="P5" s="35"/>
+      <c r="Q5" s="35"/>
+      <c r="R5" s="35"/>
+      <c r="S5" s="35"/>
+      <c r="T5" s="35"/>
+      <c r="U5" s="35"/>
+      <c r="V5" s="35"/>
+      <c r="W5" s="35"/>
+      <c r="X5" s="35"/>
+      <c r="Y5" s="35"/>
+      <c r="Z5" s="35"/>
+      <c r="AA5" s="35"/>
+      <c r="AB5" s="35"/>
+      <c r="AC5" s="35"/>
+      <c r="AD5" s="35"/>
+      <c r="AE5" s="35"/>
+      <c r="AF5" s="35"/>
+      <c r="AG5" s="36"/>
     </row>
     <row r="6" spans="1:33" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
@@ -2730,38 +2728,38 @@
       <c r="C6" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="33"/>
-      <c r="K6" s="33"/>
-      <c r="L6" s="33"/>
-      <c r="M6" s="33"/>
-      <c r="N6" s="33"/>
-      <c r="O6" s="33"/>
-      <c r="P6" s="33"/>
-      <c r="Q6" s="33"/>
-      <c r="R6" s="33"/>
-      <c r="S6" s="33"/>
-      <c r="T6" s="33"/>
-      <c r="U6" s="33"/>
-      <c r="V6" s="33"/>
-      <c r="W6" s="33"/>
-      <c r="X6" s="33"/>
-      <c r="Y6" s="33"/>
-      <c r="Z6" s="33"/>
-      <c r="AA6" s="33"/>
-      <c r="AB6" s="33"/>
-      <c r="AC6" s="33"/>
-      <c r="AD6" s="33"/>
-      <c r="AE6" s="33"/>
-      <c r="AF6" s="33"/>
-      <c r="AG6" s="34"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="35"/>
+      <c r="I6" s="35"/>
+      <c r="J6" s="35"/>
+      <c r="K6" s="35"/>
+      <c r="L6" s="35"/>
+      <c r="M6" s="35"/>
+      <c r="N6" s="35"/>
+      <c r="O6" s="35"/>
+      <c r="P6" s="35"/>
+      <c r="Q6" s="35"/>
+      <c r="R6" s="35"/>
+      <c r="S6" s="35"/>
+      <c r="T6" s="35"/>
+      <c r="U6" s="35"/>
+      <c r="V6" s="35"/>
+      <c r="W6" s="35"/>
+      <c r="X6" s="35"/>
+      <c r="Y6" s="35"/>
+      <c r="Z6" s="35"/>
+      <c r="AA6" s="35"/>
+      <c r="AB6" s="35"/>
+      <c r="AC6" s="35"/>
+      <c r="AD6" s="35"/>
+      <c r="AE6" s="35"/>
+      <c r="AF6" s="35"/>
+      <c r="AG6" s="36"/>
     </row>
     <row r="7" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="19"/>
@@ -2771,116 +2769,116 @@
       <c r="C7" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="D7" s="32" t="s">
+      <c r="D7" s="37" t="s">
         <v>557</v>
       </c>
-      <c r="E7" s="33"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="33"/>
-      <c r="I7" s="33"/>
-      <c r="J7" s="33"/>
-      <c r="K7" s="33"/>
-      <c r="L7" s="33"/>
-      <c r="M7" s="33"/>
-      <c r="N7" s="33"/>
-      <c r="O7" s="33"/>
-      <c r="P7" s="33"/>
-      <c r="Q7" s="33"/>
-      <c r="R7" s="33"/>
-      <c r="S7" s="33"/>
-      <c r="T7" s="33"/>
-      <c r="U7" s="33"/>
-      <c r="V7" s="33"/>
-      <c r="W7" s="33"/>
-      <c r="X7" s="33"/>
-      <c r="Y7" s="33"/>
-      <c r="Z7" s="33"/>
-      <c r="AA7" s="33"/>
-      <c r="AB7" s="33"/>
-      <c r="AC7" s="33"/>
-      <c r="AD7" s="33"/>
-      <c r="AE7" s="33"/>
-      <c r="AF7" s="33"/>
-      <c r="AG7" s="34"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
+      <c r="G7" s="35"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="35"/>
+      <c r="J7" s="35"/>
+      <c r="K7" s="35"/>
+      <c r="L7" s="35"/>
+      <c r="M7" s="35"/>
+      <c r="N7" s="35"/>
+      <c r="O7" s="35"/>
+      <c r="P7" s="35"/>
+      <c r="Q7" s="35"/>
+      <c r="R7" s="35"/>
+      <c r="S7" s="35"/>
+      <c r="T7" s="35"/>
+      <c r="U7" s="35"/>
+      <c r="V7" s="35"/>
+      <c r="W7" s="35"/>
+      <c r="X7" s="35"/>
+      <c r="Y7" s="35"/>
+      <c r="Z7" s="35"/>
+      <c r="AA7" s="35"/>
+      <c r="AB7" s="35"/>
+      <c r="AC7" s="35"/>
+      <c r="AD7" s="35"/>
+      <c r="AE7" s="35"/>
+      <c r="AF7" s="35"/>
+      <c r="AG7" s="36"/>
     </row>
     <row r="8" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="33"/>
-      <c r="K8" s="33"/>
-      <c r="L8" s="33"/>
-      <c r="M8" s="33"/>
-      <c r="N8" s="33"/>
-      <c r="O8" s="33"/>
-      <c r="P8" s="33"/>
-      <c r="Q8" s="33"/>
-      <c r="R8" s="33"/>
-      <c r="S8" s="33"/>
-      <c r="T8" s="33"/>
-      <c r="U8" s="33"/>
-      <c r="V8" s="33"/>
-      <c r="W8" s="33"/>
-      <c r="X8" s="33"/>
-      <c r="Y8" s="33"/>
-      <c r="Z8" s="33"/>
-      <c r="AA8" s="33"/>
-      <c r="AB8" s="33"/>
-      <c r="AC8" s="33"/>
-      <c r="AD8" s="33"/>
-      <c r="AE8" s="33"/>
-      <c r="AF8" s="33"/>
-      <c r="AG8" s="34"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="35"/>
+      <c r="K8" s="35"/>
+      <c r="L8" s="35"/>
+      <c r="M8" s="35"/>
+      <c r="N8" s="35"/>
+      <c r="O8" s="35"/>
+      <c r="P8" s="35"/>
+      <c r="Q8" s="35"/>
+      <c r="R8" s="35"/>
+      <c r="S8" s="35"/>
+      <c r="T8" s="35"/>
+      <c r="U8" s="35"/>
+      <c r="V8" s="35"/>
+      <c r="W8" s="35"/>
+      <c r="X8" s="35"/>
+      <c r="Y8" s="35"/>
+      <c r="Z8" s="35"/>
+      <c r="AA8" s="35"/>
+      <c r="AB8" s="35"/>
+      <c r="AC8" s="35"/>
+      <c r="AD8" s="35"/>
+      <c r="AE8" s="35"/>
+      <c r="AF8" s="35"/>
+      <c r="AG8" s="36"/>
     </row>
     <row r="9" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="37" t="s">
         <v>72</v>
       </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="33"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="33"/>
-      <c r="J9" s="33"/>
-      <c r="K9" s="33"/>
-      <c r="L9" s="33"/>
-      <c r="M9" s="33"/>
-      <c r="N9" s="33"/>
-      <c r="O9" s="33"/>
-      <c r="P9" s="33"/>
-      <c r="Q9" s="33"/>
-      <c r="R9" s="33"/>
-      <c r="S9" s="33"/>
-      <c r="T9" s="33"/>
-      <c r="U9" s="33"/>
-      <c r="V9" s="33"/>
-      <c r="W9" s="33"/>
-      <c r="X9" s="33"/>
-      <c r="Y9" s="33"/>
-      <c r="Z9" s="33"/>
-      <c r="AA9" s="33"/>
-      <c r="AB9" s="33"/>
-      <c r="AC9" s="33"/>
-      <c r="AD9" s="33"/>
-      <c r="AE9" s="33"/>
-      <c r="AF9" s="33"/>
-      <c r="AG9" s="34"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="35"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="35"/>
+      <c r="J9" s="35"/>
+      <c r="K9" s="35"/>
+      <c r="L9" s="35"/>
+      <c r="M9" s="35"/>
+      <c r="N9" s="35"/>
+      <c r="O9" s="35"/>
+      <c r="P9" s="35"/>
+      <c r="Q9" s="35"/>
+      <c r="R9" s="35"/>
+      <c r="S9" s="35"/>
+      <c r="T9" s="35"/>
+      <c r="U9" s="35"/>
+      <c r="V9" s="35"/>
+      <c r="W9" s="35"/>
+      <c r="X9" s="35"/>
+      <c r="Y9" s="35"/>
+      <c r="Z9" s="35"/>
+      <c r="AA9" s="35"/>
+      <c r="AB9" s="35"/>
+      <c r="AC9" s="35"/>
+      <c r="AD9" s="35"/>
+      <c r="AE9" s="35"/>
+      <c r="AF9" s="35"/>
+      <c r="AG9" s="36"/>
     </row>
     <row r="10" spans="1:33" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="23" t="s">
@@ -3769,79 +3767,79 @@
       <c r="A26" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B26" s="36" t="s">
+      <c r="B26" s="38" t="s">
         <v>230</v>
       </c>
-      <c r="C26" s="33"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="33"/>
-      <c r="J26" s="33"/>
-      <c r="K26" s="33"/>
-      <c r="L26" s="33"/>
-      <c r="M26" s="33"/>
-      <c r="N26" s="33"/>
-      <c r="O26" s="33"/>
-      <c r="P26" s="33"/>
-      <c r="Q26" s="33"/>
-      <c r="R26" s="33"/>
-      <c r="S26" s="33"/>
-      <c r="T26" s="33"/>
-      <c r="U26" s="33"/>
-      <c r="V26" s="33"/>
-      <c r="W26" s="33"/>
-      <c r="X26" s="33"/>
-      <c r="Y26" s="33"/>
-      <c r="Z26" s="33"/>
-      <c r="AA26" s="33"/>
-      <c r="AB26" s="33"/>
-      <c r="AC26" s="33"/>
-      <c r="AD26" s="33"/>
-      <c r="AE26" s="33"/>
-      <c r="AF26" s="33"/>
-      <c r="AG26" s="34"/>
+      <c r="C26" s="35"/>
+      <c r="D26" s="35"/>
+      <c r="E26" s="35"/>
+      <c r="F26" s="35"/>
+      <c r="G26" s="35"/>
+      <c r="H26" s="35"/>
+      <c r="I26" s="35"/>
+      <c r="J26" s="35"/>
+      <c r="K26" s="35"/>
+      <c r="L26" s="35"/>
+      <c r="M26" s="35"/>
+      <c r="N26" s="35"/>
+      <c r="O26" s="35"/>
+      <c r="P26" s="35"/>
+      <c r="Q26" s="35"/>
+      <c r="R26" s="35"/>
+      <c r="S26" s="35"/>
+      <c r="T26" s="35"/>
+      <c r="U26" s="35"/>
+      <c r="V26" s="35"/>
+      <c r="W26" s="35"/>
+      <c r="X26" s="35"/>
+      <c r="Y26" s="35"/>
+      <c r="Z26" s="35"/>
+      <c r="AA26" s="35"/>
+      <c r="AB26" s="35"/>
+      <c r="AC26" s="35"/>
+      <c r="AD26" s="35"/>
+      <c r="AE26" s="35"/>
+      <c r="AF26" s="35"/>
+      <c r="AG26" s="36"/>
     </row>
     <row r="27" spans="1:33" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="B27" s="32" t="s">
+      <c r="B27" s="37" t="s">
         <v>231</v>
       </c>
-      <c r="C27" s="33"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="33"/>
-      <c r="J27" s="33"/>
-      <c r="K27" s="33"/>
-      <c r="L27" s="33"/>
-      <c r="M27" s="33"/>
-      <c r="N27" s="33"/>
-      <c r="O27" s="33"/>
-      <c r="P27" s="33"/>
-      <c r="Q27" s="33"/>
-      <c r="R27" s="33"/>
-      <c r="S27" s="33"/>
-      <c r="T27" s="33"/>
-      <c r="U27" s="33"/>
-      <c r="V27" s="33"/>
-      <c r="W27" s="33"/>
-      <c r="X27" s="33"/>
-      <c r="Y27" s="33"/>
-      <c r="Z27" s="33"/>
-      <c r="AA27" s="33"/>
-      <c r="AB27" s="33"/>
-      <c r="AC27" s="33"/>
-      <c r="AD27" s="33"/>
-      <c r="AE27" s="33"/>
-      <c r="AF27" s="33"/>
-      <c r="AG27" s="34"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35"/>
+      <c r="H27" s="35"/>
+      <c r="I27" s="35"/>
+      <c r="J27" s="35"/>
+      <c r="K27" s="35"/>
+      <c r="L27" s="35"/>
+      <c r="M27" s="35"/>
+      <c r="N27" s="35"/>
+      <c r="O27" s="35"/>
+      <c r="P27" s="35"/>
+      <c r="Q27" s="35"/>
+      <c r="R27" s="35"/>
+      <c r="S27" s="35"/>
+      <c r="T27" s="35"/>
+      <c r="U27" s="35"/>
+      <c r="V27" s="35"/>
+      <c r="W27" s="35"/>
+      <c r="X27" s="35"/>
+      <c r="Y27" s="35"/>
+      <c r="Z27" s="35"/>
+      <c r="AA27" s="35"/>
+      <c r="AB27" s="35"/>
+      <c r="AC27" s="35"/>
+      <c r="AD27" s="35"/>
+      <c r="AE27" s="35"/>
+      <c r="AF27" s="35"/>
+      <c r="AG27" s="36"/>
     </row>
     <row r="28" spans="1:33" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="19" t="s">
@@ -3853,38 +3851,38 @@
       <c r="C28" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="35" t="s">
+      <c r="D28" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="33"/>
-      <c r="K28" s="33"/>
-      <c r="L28" s="33"/>
-      <c r="M28" s="33"/>
-      <c r="N28" s="33"/>
-      <c r="O28" s="33"/>
-      <c r="P28" s="33"/>
-      <c r="Q28" s="33"/>
-      <c r="R28" s="33"/>
-      <c r="S28" s="33"/>
-      <c r="T28" s="33"/>
-      <c r="U28" s="33"/>
-      <c r="V28" s="33"/>
-      <c r="W28" s="33"/>
-      <c r="X28" s="33"/>
-      <c r="Y28" s="33"/>
-      <c r="Z28" s="33"/>
-      <c r="AA28" s="33"/>
-      <c r="AB28" s="33"/>
-      <c r="AC28" s="33"/>
-      <c r="AD28" s="33"/>
-      <c r="AE28" s="33"/>
-      <c r="AF28" s="33"/>
-      <c r="AG28" s="34"/>
+      <c r="E28" s="35"/>
+      <c r="F28" s="35"/>
+      <c r="G28" s="35"/>
+      <c r="H28" s="35"/>
+      <c r="I28" s="35"/>
+      <c r="J28" s="35"/>
+      <c r="K28" s="35"/>
+      <c r="L28" s="35"/>
+      <c r="M28" s="35"/>
+      <c r="N28" s="35"/>
+      <c r="O28" s="35"/>
+      <c r="P28" s="35"/>
+      <c r="Q28" s="35"/>
+      <c r="R28" s="35"/>
+      <c r="S28" s="35"/>
+      <c r="T28" s="35"/>
+      <c r="U28" s="35"/>
+      <c r="V28" s="35"/>
+      <c r="W28" s="35"/>
+      <c r="X28" s="35"/>
+      <c r="Y28" s="35"/>
+      <c r="Z28" s="35"/>
+      <c r="AA28" s="35"/>
+      <c r="AB28" s="35"/>
+      <c r="AC28" s="35"/>
+      <c r="AD28" s="35"/>
+      <c r="AE28" s="35"/>
+      <c r="AF28" s="35"/>
+      <c r="AG28" s="36"/>
     </row>
     <row r="29" spans="1:33" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="19"/>
@@ -3894,116 +3892,116 @@
       <c r="C29" s="21" t="s">
         <v>232</v>
       </c>
-      <c r="D29" s="32" t="s">
+      <c r="D29" s="37" t="s">
         <v>233</v>
       </c>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="33"/>
-      <c r="I29" s="33"/>
-      <c r="J29" s="33"/>
-      <c r="K29" s="33"/>
-      <c r="L29" s="33"/>
-      <c r="M29" s="33"/>
-      <c r="N29" s="33"/>
-      <c r="O29" s="33"/>
-      <c r="P29" s="33"/>
-      <c r="Q29" s="33"/>
-      <c r="R29" s="33"/>
-      <c r="S29" s="33"/>
-      <c r="T29" s="33"/>
-      <c r="U29" s="33"/>
-      <c r="V29" s="33"/>
-      <c r="W29" s="33"/>
-      <c r="X29" s="33"/>
-      <c r="Y29" s="33"/>
-      <c r="Z29" s="33"/>
-      <c r="AA29" s="33"/>
-      <c r="AB29" s="33"/>
-      <c r="AC29" s="33"/>
-      <c r="AD29" s="33"/>
-      <c r="AE29" s="33"/>
-      <c r="AF29" s="33"/>
-      <c r="AG29" s="34"/>
+      <c r="E29" s="35"/>
+      <c r="F29" s="35"/>
+      <c r="G29" s="35"/>
+      <c r="H29" s="35"/>
+      <c r="I29" s="35"/>
+      <c r="J29" s="35"/>
+      <c r="K29" s="35"/>
+      <c r="L29" s="35"/>
+      <c r="M29" s="35"/>
+      <c r="N29" s="35"/>
+      <c r="O29" s="35"/>
+      <c r="P29" s="35"/>
+      <c r="Q29" s="35"/>
+      <c r="R29" s="35"/>
+      <c r="S29" s="35"/>
+      <c r="T29" s="35"/>
+      <c r="U29" s="35"/>
+      <c r="V29" s="35"/>
+      <c r="W29" s="35"/>
+      <c r="X29" s="35"/>
+      <c r="Y29" s="35"/>
+      <c r="Z29" s="35"/>
+      <c r="AA29" s="35"/>
+      <c r="AB29" s="35"/>
+      <c r="AC29" s="35"/>
+      <c r="AD29" s="35"/>
+      <c r="AE29" s="35"/>
+      <c r="AF29" s="35"/>
+      <c r="AG29" s="36"/>
     </row>
     <row r="30" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="B30" s="36" t="s">
+      <c r="B30" s="38" t="s">
         <v>234</v>
       </c>
-      <c r="C30" s="33"/>
-      <c r="D30" s="33"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="33"/>
-      <c r="G30" s="33"/>
-      <c r="H30" s="33"/>
-      <c r="I30" s="33"/>
-      <c r="J30" s="33"/>
-      <c r="K30" s="33"/>
-      <c r="L30" s="33"/>
-      <c r="M30" s="33"/>
-      <c r="N30" s="33"/>
-      <c r="O30" s="33"/>
-      <c r="P30" s="33"/>
-      <c r="Q30" s="33"/>
-      <c r="R30" s="33"/>
-      <c r="S30" s="33"/>
-      <c r="T30" s="33"/>
-      <c r="U30" s="33"/>
-      <c r="V30" s="33"/>
-      <c r="W30" s="33"/>
-      <c r="X30" s="33"/>
-      <c r="Y30" s="33"/>
-      <c r="Z30" s="33"/>
-      <c r="AA30" s="33"/>
-      <c r="AB30" s="33"/>
-      <c r="AC30" s="33"/>
-      <c r="AD30" s="33"/>
-      <c r="AE30" s="33"/>
-      <c r="AF30" s="33"/>
-      <c r="AG30" s="34"/>
+      <c r="C30" s="35"/>
+      <c r="D30" s="35"/>
+      <c r="E30" s="35"/>
+      <c r="F30" s="35"/>
+      <c r="G30" s="35"/>
+      <c r="H30" s="35"/>
+      <c r="I30" s="35"/>
+      <c r="J30" s="35"/>
+      <c r="K30" s="35"/>
+      <c r="L30" s="35"/>
+      <c r="M30" s="35"/>
+      <c r="N30" s="35"/>
+      <c r="O30" s="35"/>
+      <c r="P30" s="35"/>
+      <c r="Q30" s="35"/>
+      <c r="R30" s="35"/>
+      <c r="S30" s="35"/>
+      <c r="T30" s="35"/>
+      <c r="U30" s="35"/>
+      <c r="V30" s="35"/>
+      <c r="W30" s="35"/>
+      <c r="X30" s="35"/>
+      <c r="Y30" s="35"/>
+      <c r="Z30" s="35"/>
+      <c r="AA30" s="35"/>
+      <c r="AB30" s="35"/>
+      <c r="AC30" s="35"/>
+      <c r="AD30" s="35"/>
+      <c r="AE30" s="35"/>
+      <c r="AF30" s="35"/>
+      <c r="AG30" s="36"/>
     </row>
     <row r="31" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="B31" s="32" t="s">
+      <c r="B31" s="37" t="s">
         <v>235</v>
       </c>
-      <c r="C31" s="33"/>
-      <c r="D31" s="33"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="33"/>
-      <c r="G31" s="33"/>
-      <c r="H31" s="33"/>
-      <c r="I31" s="33"/>
-      <c r="J31" s="33"/>
-      <c r="K31" s="33"/>
-      <c r="L31" s="33"/>
-      <c r="M31" s="33"/>
-      <c r="N31" s="33"/>
-      <c r="O31" s="33"/>
-      <c r="P31" s="33"/>
-      <c r="Q31" s="33"/>
-      <c r="R31" s="33"/>
-      <c r="S31" s="33"/>
-      <c r="T31" s="33"/>
-      <c r="U31" s="33"/>
-      <c r="V31" s="33"/>
-      <c r="W31" s="33"/>
-      <c r="X31" s="33"/>
-      <c r="Y31" s="33"/>
-      <c r="Z31" s="33"/>
-      <c r="AA31" s="33"/>
-      <c r="AB31" s="33"/>
-      <c r="AC31" s="33"/>
-      <c r="AD31" s="33"/>
-      <c r="AE31" s="33"/>
-      <c r="AF31" s="33"/>
-      <c r="AG31" s="34"/>
+      <c r="C31" s="35"/>
+      <c r="D31" s="35"/>
+      <c r="E31" s="35"/>
+      <c r="F31" s="35"/>
+      <c r="G31" s="35"/>
+      <c r="H31" s="35"/>
+      <c r="I31" s="35"/>
+      <c r="J31" s="35"/>
+      <c r="K31" s="35"/>
+      <c r="L31" s="35"/>
+      <c r="M31" s="35"/>
+      <c r="N31" s="35"/>
+      <c r="O31" s="35"/>
+      <c r="P31" s="35"/>
+      <c r="Q31" s="35"/>
+      <c r="R31" s="35"/>
+      <c r="S31" s="35"/>
+      <c r="T31" s="35"/>
+      <c r="U31" s="35"/>
+      <c r="V31" s="35"/>
+      <c r="W31" s="35"/>
+      <c r="X31" s="35"/>
+      <c r="Y31" s="35"/>
+      <c r="Z31" s="35"/>
+      <c r="AA31" s="35"/>
+      <c r="AB31" s="35"/>
+      <c r="AC31" s="35"/>
+      <c r="AD31" s="35"/>
+      <c r="AE31" s="35"/>
+      <c r="AF31" s="35"/>
+      <c r="AG31" s="36"/>
     </row>
     <row r="32" spans="1:33" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="23" t="s">
@@ -4999,79 +4997,79 @@
       <c r="A48" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B48" s="36" t="s">
+      <c r="B48" s="38" t="s">
         <v>372</v>
       </c>
-      <c r="C48" s="33"/>
-      <c r="D48" s="33"/>
-      <c r="E48" s="33"/>
-      <c r="F48" s="33"/>
-      <c r="G48" s="33"/>
-      <c r="H48" s="33"/>
-      <c r="I48" s="33"/>
-      <c r="J48" s="33"/>
-      <c r="K48" s="33"/>
-      <c r="L48" s="33"/>
-      <c r="M48" s="33"/>
-      <c r="N48" s="33"/>
-      <c r="O48" s="33"/>
-      <c r="P48" s="33"/>
-      <c r="Q48" s="33"/>
-      <c r="R48" s="33"/>
-      <c r="S48" s="33"/>
-      <c r="T48" s="33"/>
-      <c r="U48" s="33"/>
-      <c r="V48" s="33"/>
-      <c r="W48" s="33"/>
-      <c r="X48" s="33"/>
-      <c r="Y48" s="33"/>
-      <c r="Z48" s="33"/>
-      <c r="AA48" s="33"/>
-      <c r="AB48" s="33"/>
-      <c r="AC48" s="33"/>
-      <c r="AD48" s="33"/>
-      <c r="AE48" s="33"/>
-      <c r="AF48" s="33"/>
-      <c r="AG48" s="34"/>
+      <c r="C48" s="35"/>
+      <c r="D48" s="35"/>
+      <c r="E48" s="35"/>
+      <c r="F48" s="35"/>
+      <c r="G48" s="35"/>
+      <c r="H48" s="35"/>
+      <c r="I48" s="35"/>
+      <c r="J48" s="35"/>
+      <c r="K48" s="35"/>
+      <c r="L48" s="35"/>
+      <c r="M48" s="35"/>
+      <c r="N48" s="35"/>
+      <c r="O48" s="35"/>
+      <c r="P48" s="35"/>
+      <c r="Q48" s="35"/>
+      <c r="R48" s="35"/>
+      <c r="S48" s="35"/>
+      <c r="T48" s="35"/>
+      <c r="U48" s="35"/>
+      <c r="V48" s="35"/>
+      <c r="W48" s="35"/>
+      <c r="X48" s="35"/>
+      <c r="Y48" s="35"/>
+      <c r="Z48" s="35"/>
+      <c r="AA48" s="35"/>
+      <c r="AB48" s="35"/>
+      <c r="AC48" s="35"/>
+      <c r="AD48" s="35"/>
+      <c r="AE48" s="35"/>
+      <c r="AF48" s="35"/>
+      <c r="AG48" s="36"/>
     </row>
     <row r="49" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="B49" s="32" t="s">
+      <c r="B49" s="37" t="s">
         <v>373</v>
       </c>
-      <c r="C49" s="33"/>
-      <c r="D49" s="33"/>
-      <c r="E49" s="33"/>
-      <c r="F49" s="33"/>
-      <c r="G49" s="33"/>
-      <c r="H49" s="33"/>
-      <c r="I49" s="33"/>
-      <c r="J49" s="33"/>
-      <c r="K49" s="33"/>
-      <c r="L49" s="33"/>
-      <c r="M49" s="33"/>
-      <c r="N49" s="33"/>
-      <c r="O49" s="33"/>
-      <c r="P49" s="33"/>
-      <c r="Q49" s="33"/>
-      <c r="R49" s="33"/>
-      <c r="S49" s="33"/>
-      <c r="T49" s="33"/>
-      <c r="U49" s="33"/>
-      <c r="V49" s="33"/>
-      <c r="W49" s="33"/>
-      <c r="X49" s="33"/>
-      <c r="Y49" s="33"/>
-      <c r="Z49" s="33"/>
-      <c r="AA49" s="33"/>
-      <c r="AB49" s="33"/>
-      <c r="AC49" s="33"/>
-      <c r="AD49" s="33"/>
-      <c r="AE49" s="33"/>
-      <c r="AF49" s="33"/>
-      <c r="AG49" s="34"/>
+      <c r="C49" s="35"/>
+      <c r="D49" s="35"/>
+      <c r="E49" s="35"/>
+      <c r="F49" s="35"/>
+      <c r="G49" s="35"/>
+      <c r="H49" s="35"/>
+      <c r="I49" s="35"/>
+      <c r="J49" s="35"/>
+      <c r="K49" s="35"/>
+      <c r="L49" s="35"/>
+      <c r="M49" s="35"/>
+      <c r="N49" s="35"/>
+      <c r="O49" s="35"/>
+      <c r="P49" s="35"/>
+      <c r="Q49" s="35"/>
+      <c r="R49" s="35"/>
+      <c r="S49" s="35"/>
+      <c r="T49" s="35"/>
+      <c r="U49" s="35"/>
+      <c r="V49" s="35"/>
+      <c r="W49" s="35"/>
+      <c r="X49" s="35"/>
+      <c r="Y49" s="35"/>
+      <c r="Z49" s="35"/>
+      <c r="AA49" s="35"/>
+      <c r="AB49" s="35"/>
+      <c r="AC49" s="35"/>
+      <c r="AD49" s="35"/>
+      <c r="AE49" s="35"/>
+      <c r="AF49" s="35"/>
+      <c r="AG49" s="36"/>
     </row>
     <row r="50" spans="1:33" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="19" t="s">
@@ -5083,38 +5081,38 @@
       <c r="C50" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="D50" s="35" t="s">
+      <c r="D50" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="E50" s="33"/>
-      <c r="F50" s="33"/>
-      <c r="G50" s="33"/>
-      <c r="H50" s="33"/>
-      <c r="I50" s="33"/>
-      <c r="J50" s="33"/>
-      <c r="K50" s="33"/>
-      <c r="L50" s="33"/>
-      <c r="M50" s="33"/>
-      <c r="N50" s="33"/>
-      <c r="O50" s="33"/>
-      <c r="P50" s="33"/>
-      <c r="Q50" s="33"/>
-      <c r="R50" s="33"/>
-      <c r="S50" s="33"/>
-      <c r="T50" s="33"/>
-      <c r="U50" s="33"/>
-      <c r="V50" s="33"/>
-      <c r="W50" s="33"/>
-      <c r="X50" s="33"/>
-      <c r="Y50" s="33"/>
-      <c r="Z50" s="33"/>
-      <c r="AA50" s="33"/>
-      <c r="AB50" s="33"/>
-      <c r="AC50" s="33"/>
-      <c r="AD50" s="33"/>
-      <c r="AE50" s="33"/>
-      <c r="AF50" s="33"/>
-      <c r="AG50" s="34"/>
+      <c r="E50" s="35"/>
+      <c r="F50" s="35"/>
+      <c r="G50" s="35"/>
+      <c r="H50" s="35"/>
+      <c r="I50" s="35"/>
+      <c r="J50" s="35"/>
+      <c r="K50" s="35"/>
+      <c r="L50" s="35"/>
+      <c r="M50" s="35"/>
+      <c r="N50" s="35"/>
+      <c r="O50" s="35"/>
+      <c r="P50" s="35"/>
+      <c r="Q50" s="35"/>
+      <c r="R50" s="35"/>
+      <c r="S50" s="35"/>
+      <c r="T50" s="35"/>
+      <c r="U50" s="35"/>
+      <c r="V50" s="35"/>
+      <c r="W50" s="35"/>
+      <c r="X50" s="35"/>
+      <c r="Y50" s="35"/>
+      <c r="Z50" s="35"/>
+      <c r="AA50" s="35"/>
+      <c r="AB50" s="35"/>
+      <c r="AC50" s="35"/>
+      <c r="AD50" s="35"/>
+      <c r="AE50" s="35"/>
+      <c r="AF50" s="35"/>
+      <c r="AG50" s="36"/>
     </row>
     <row r="51" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="19"/>
@@ -5124,116 +5122,116 @@
       <c r="C51" s="21" t="s">
         <v>374</v>
       </c>
-      <c r="D51" s="32" t="s">
+      <c r="D51" s="37" t="s">
         <v>375</v>
       </c>
-      <c r="E51" s="33"/>
-      <c r="F51" s="33"/>
-      <c r="G51" s="33"/>
-      <c r="H51" s="33"/>
-      <c r="I51" s="33"/>
-      <c r="J51" s="33"/>
-      <c r="K51" s="33"/>
-      <c r="L51" s="33"/>
-      <c r="M51" s="33"/>
-      <c r="N51" s="33"/>
-      <c r="O51" s="33"/>
-      <c r="P51" s="33"/>
-      <c r="Q51" s="33"/>
-      <c r="R51" s="33"/>
-      <c r="S51" s="33"/>
-      <c r="T51" s="33"/>
-      <c r="U51" s="33"/>
-      <c r="V51" s="33"/>
-      <c r="W51" s="33"/>
-      <c r="X51" s="33"/>
-      <c r="Y51" s="33"/>
-      <c r="Z51" s="33"/>
-      <c r="AA51" s="33"/>
-      <c r="AB51" s="33"/>
-      <c r="AC51" s="33"/>
-      <c r="AD51" s="33"/>
-      <c r="AE51" s="33"/>
-      <c r="AF51" s="33"/>
-      <c r="AG51" s="34"/>
+      <c r="E51" s="35"/>
+      <c r="F51" s="35"/>
+      <c r="G51" s="35"/>
+      <c r="H51" s="35"/>
+      <c r="I51" s="35"/>
+      <c r="J51" s="35"/>
+      <c r="K51" s="35"/>
+      <c r="L51" s="35"/>
+      <c r="M51" s="35"/>
+      <c r="N51" s="35"/>
+      <c r="O51" s="35"/>
+      <c r="P51" s="35"/>
+      <c r="Q51" s="35"/>
+      <c r="R51" s="35"/>
+      <c r="S51" s="35"/>
+      <c r="T51" s="35"/>
+      <c r="U51" s="35"/>
+      <c r="V51" s="35"/>
+      <c r="W51" s="35"/>
+      <c r="X51" s="35"/>
+      <c r="Y51" s="35"/>
+      <c r="Z51" s="35"/>
+      <c r="AA51" s="35"/>
+      <c r="AB51" s="35"/>
+      <c r="AC51" s="35"/>
+      <c r="AD51" s="35"/>
+      <c r="AE51" s="35"/>
+      <c r="AF51" s="35"/>
+      <c r="AG51" s="36"/>
     </row>
     <row r="52" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="B52" s="36" t="s">
+      <c r="B52" s="38" t="s">
         <v>376</v>
       </c>
-      <c r="C52" s="33"/>
-      <c r="D52" s="33"/>
-      <c r="E52" s="33"/>
-      <c r="F52" s="33"/>
-      <c r="G52" s="33"/>
-      <c r="H52" s="33"/>
-      <c r="I52" s="33"/>
-      <c r="J52" s="33"/>
-      <c r="K52" s="33"/>
-      <c r="L52" s="33"/>
-      <c r="M52" s="33"/>
-      <c r="N52" s="33"/>
-      <c r="O52" s="33"/>
-      <c r="P52" s="33"/>
-      <c r="Q52" s="33"/>
-      <c r="R52" s="33"/>
-      <c r="S52" s="33"/>
-      <c r="T52" s="33"/>
-      <c r="U52" s="33"/>
-      <c r="V52" s="33"/>
-      <c r="W52" s="33"/>
-      <c r="X52" s="33"/>
-      <c r="Y52" s="33"/>
-      <c r="Z52" s="33"/>
-      <c r="AA52" s="33"/>
-      <c r="AB52" s="33"/>
-      <c r="AC52" s="33"/>
-      <c r="AD52" s="33"/>
-      <c r="AE52" s="33"/>
-      <c r="AF52" s="33"/>
-      <c r="AG52" s="34"/>
+      <c r="C52" s="35"/>
+      <c r="D52" s="35"/>
+      <c r="E52" s="35"/>
+      <c r="F52" s="35"/>
+      <c r="G52" s="35"/>
+      <c r="H52" s="35"/>
+      <c r="I52" s="35"/>
+      <c r="J52" s="35"/>
+      <c r="K52" s="35"/>
+      <c r="L52" s="35"/>
+      <c r="M52" s="35"/>
+      <c r="N52" s="35"/>
+      <c r="O52" s="35"/>
+      <c r="P52" s="35"/>
+      <c r="Q52" s="35"/>
+      <c r="R52" s="35"/>
+      <c r="S52" s="35"/>
+      <c r="T52" s="35"/>
+      <c r="U52" s="35"/>
+      <c r="V52" s="35"/>
+      <c r="W52" s="35"/>
+      <c r="X52" s="35"/>
+      <c r="Y52" s="35"/>
+      <c r="Z52" s="35"/>
+      <c r="AA52" s="35"/>
+      <c r="AB52" s="35"/>
+      <c r="AC52" s="35"/>
+      <c r="AD52" s="35"/>
+      <c r="AE52" s="35"/>
+      <c r="AF52" s="35"/>
+      <c r="AG52" s="36"/>
     </row>
     <row r="53" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="B53" s="32" t="s">
+      <c r="B53" s="37" t="s">
         <v>377</v>
       </c>
-      <c r="C53" s="33"/>
-      <c r="D53" s="33"/>
-      <c r="E53" s="33"/>
-      <c r="F53" s="33"/>
-      <c r="G53" s="33"/>
-      <c r="H53" s="33"/>
-      <c r="I53" s="33"/>
-      <c r="J53" s="33"/>
-      <c r="K53" s="33"/>
-      <c r="L53" s="33"/>
-      <c r="M53" s="33"/>
-      <c r="N53" s="33"/>
-      <c r="O53" s="33"/>
-      <c r="P53" s="33"/>
-      <c r="Q53" s="33"/>
-      <c r="R53" s="33"/>
-      <c r="S53" s="33"/>
-      <c r="T53" s="33"/>
-      <c r="U53" s="33"/>
-      <c r="V53" s="33"/>
-      <c r="W53" s="33"/>
-      <c r="X53" s="33"/>
-      <c r="Y53" s="33"/>
-      <c r="Z53" s="33"/>
-      <c r="AA53" s="33"/>
-      <c r="AB53" s="33"/>
-      <c r="AC53" s="33"/>
-      <c r="AD53" s="33"/>
-      <c r="AE53" s="33"/>
-      <c r="AF53" s="33"/>
-      <c r="AG53" s="34"/>
+      <c r="C53" s="35"/>
+      <c r="D53" s="35"/>
+      <c r="E53" s="35"/>
+      <c r="F53" s="35"/>
+      <c r="G53" s="35"/>
+      <c r="H53" s="35"/>
+      <c r="I53" s="35"/>
+      <c r="J53" s="35"/>
+      <c r="K53" s="35"/>
+      <c r="L53" s="35"/>
+      <c r="M53" s="35"/>
+      <c r="N53" s="35"/>
+      <c r="O53" s="35"/>
+      <c r="P53" s="35"/>
+      <c r="Q53" s="35"/>
+      <c r="R53" s="35"/>
+      <c r="S53" s="35"/>
+      <c r="T53" s="35"/>
+      <c r="U53" s="35"/>
+      <c r="V53" s="35"/>
+      <c r="W53" s="35"/>
+      <c r="X53" s="35"/>
+      <c r="Y53" s="35"/>
+      <c r="Z53" s="35"/>
+      <c r="AA53" s="35"/>
+      <c r="AB53" s="35"/>
+      <c r="AC53" s="35"/>
+      <c r="AD53" s="35"/>
+      <c r="AE53" s="35"/>
+      <c r="AF53" s="35"/>
+      <c r="AG53" s="36"/>
     </row>
     <row r="54" spans="1:33" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="23" t="s">
@@ -5527,79 +5525,79 @@
       <c r="A70" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B70" s="36" t="s">
+      <c r="B70" s="38" t="s">
         <v>406</v>
       </c>
-      <c r="C70" s="33"/>
-      <c r="D70" s="33"/>
-      <c r="E70" s="33"/>
-      <c r="F70" s="33"/>
-      <c r="G70" s="33"/>
-      <c r="H70" s="33"/>
-      <c r="I70" s="33"/>
-      <c r="J70" s="33"/>
-      <c r="K70" s="33"/>
-      <c r="L70" s="33"/>
-      <c r="M70" s="33"/>
-      <c r="N70" s="33"/>
-      <c r="O70" s="33"/>
-      <c r="P70" s="33"/>
-      <c r="Q70" s="33"/>
-      <c r="R70" s="33"/>
-      <c r="S70" s="33"/>
-      <c r="T70" s="33"/>
-      <c r="U70" s="33"/>
-      <c r="V70" s="33"/>
-      <c r="W70" s="33"/>
-      <c r="X70" s="33"/>
-      <c r="Y70" s="33"/>
-      <c r="Z70" s="33"/>
-      <c r="AA70" s="33"/>
-      <c r="AB70" s="33"/>
-      <c r="AC70" s="33"/>
-      <c r="AD70" s="33"/>
-      <c r="AE70" s="33"/>
-      <c r="AF70" s="33"/>
-      <c r="AG70" s="34"/>
+      <c r="C70" s="35"/>
+      <c r="D70" s="35"/>
+      <c r="E70" s="35"/>
+      <c r="F70" s="35"/>
+      <c r="G70" s="35"/>
+      <c r="H70" s="35"/>
+      <c r="I70" s="35"/>
+      <c r="J70" s="35"/>
+      <c r="K70" s="35"/>
+      <c r="L70" s="35"/>
+      <c r="M70" s="35"/>
+      <c r="N70" s="35"/>
+      <c r="O70" s="35"/>
+      <c r="P70" s="35"/>
+      <c r="Q70" s="35"/>
+      <c r="R70" s="35"/>
+      <c r="S70" s="35"/>
+      <c r="T70" s="35"/>
+      <c r="U70" s="35"/>
+      <c r="V70" s="35"/>
+      <c r="W70" s="35"/>
+      <c r="X70" s="35"/>
+      <c r="Y70" s="35"/>
+      <c r="Z70" s="35"/>
+      <c r="AA70" s="35"/>
+      <c r="AB70" s="35"/>
+      <c r="AC70" s="35"/>
+      <c r="AD70" s="35"/>
+      <c r="AE70" s="35"/>
+      <c r="AF70" s="35"/>
+      <c r="AG70" s="36"/>
     </row>
     <row r="71" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="B71" s="32" t="s">
+      <c r="B71" s="37" t="s">
         <v>407</v>
       </c>
-      <c r="C71" s="33"/>
-      <c r="D71" s="33"/>
-      <c r="E71" s="33"/>
-      <c r="F71" s="33"/>
-      <c r="G71" s="33"/>
-      <c r="H71" s="33"/>
-      <c r="I71" s="33"/>
-      <c r="J71" s="33"/>
-      <c r="K71" s="33"/>
-      <c r="L71" s="33"/>
-      <c r="M71" s="33"/>
-      <c r="N71" s="33"/>
-      <c r="O71" s="33"/>
-      <c r="P71" s="33"/>
-      <c r="Q71" s="33"/>
-      <c r="R71" s="33"/>
-      <c r="S71" s="33"/>
-      <c r="T71" s="33"/>
-      <c r="U71" s="33"/>
-      <c r="V71" s="33"/>
-      <c r="W71" s="33"/>
-      <c r="X71" s="33"/>
-      <c r="Y71" s="33"/>
-      <c r="Z71" s="33"/>
-      <c r="AA71" s="33"/>
-      <c r="AB71" s="33"/>
-      <c r="AC71" s="33"/>
-      <c r="AD71" s="33"/>
-      <c r="AE71" s="33"/>
-      <c r="AF71" s="33"/>
-      <c r="AG71" s="34"/>
+      <c r="C71" s="35"/>
+      <c r="D71" s="35"/>
+      <c r="E71" s="35"/>
+      <c r="F71" s="35"/>
+      <c r="G71" s="35"/>
+      <c r="H71" s="35"/>
+      <c r="I71" s="35"/>
+      <c r="J71" s="35"/>
+      <c r="K71" s="35"/>
+      <c r="L71" s="35"/>
+      <c r="M71" s="35"/>
+      <c r="N71" s="35"/>
+      <c r="O71" s="35"/>
+      <c r="P71" s="35"/>
+      <c r="Q71" s="35"/>
+      <c r="R71" s="35"/>
+      <c r="S71" s="35"/>
+      <c r="T71" s="35"/>
+      <c r="U71" s="35"/>
+      <c r="V71" s="35"/>
+      <c r="W71" s="35"/>
+      <c r="X71" s="35"/>
+      <c r="Y71" s="35"/>
+      <c r="Z71" s="35"/>
+      <c r="AA71" s="35"/>
+      <c r="AB71" s="35"/>
+      <c r="AC71" s="35"/>
+      <c r="AD71" s="35"/>
+      <c r="AE71" s="35"/>
+      <c r="AF71" s="35"/>
+      <c r="AG71" s="36"/>
     </row>
     <row r="72" spans="1:33" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="19" t="s">
@@ -5611,38 +5609,38 @@
       <c r="C72" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="D72" s="35" t="s">
+      <c r="D72" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="E72" s="33"/>
-      <c r="F72" s="33"/>
-      <c r="G72" s="33"/>
-      <c r="H72" s="33"/>
-      <c r="I72" s="33"/>
-      <c r="J72" s="33"/>
-      <c r="K72" s="33"/>
-      <c r="L72" s="33"/>
-      <c r="M72" s="33"/>
-      <c r="N72" s="33"/>
-      <c r="O72" s="33"/>
-      <c r="P72" s="33"/>
-      <c r="Q72" s="33"/>
-      <c r="R72" s="33"/>
-      <c r="S72" s="33"/>
-      <c r="T72" s="33"/>
-      <c r="U72" s="33"/>
-      <c r="V72" s="33"/>
-      <c r="W72" s="33"/>
-      <c r="X72" s="33"/>
-      <c r="Y72" s="33"/>
-      <c r="Z72" s="33"/>
-      <c r="AA72" s="33"/>
-      <c r="AB72" s="33"/>
-      <c r="AC72" s="33"/>
-      <c r="AD72" s="33"/>
-      <c r="AE72" s="33"/>
-      <c r="AF72" s="33"/>
-      <c r="AG72" s="34"/>
+      <c r="E72" s="35"/>
+      <c r="F72" s="35"/>
+      <c r="G72" s="35"/>
+      <c r="H72" s="35"/>
+      <c r="I72" s="35"/>
+      <c r="J72" s="35"/>
+      <c r="K72" s="35"/>
+      <c r="L72" s="35"/>
+      <c r="M72" s="35"/>
+      <c r="N72" s="35"/>
+      <c r="O72" s="35"/>
+      <c r="P72" s="35"/>
+      <c r="Q72" s="35"/>
+      <c r="R72" s="35"/>
+      <c r="S72" s="35"/>
+      <c r="T72" s="35"/>
+      <c r="U72" s="35"/>
+      <c r="V72" s="35"/>
+      <c r="W72" s="35"/>
+      <c r="X72" s="35"/>
+      <c r="Y72" s="35"/>
+      <c r="Z72" s="35"/>
+      <c r="AA72" s="35"/>
+      <c r="AB72" s="35"/>
+      <c r="AC72" s="35"/>
+      <c r="AD72" s="35"/>
+      <c r="AE72" s="35"/>
+      <c r="AF72" s="35"/>
+      <c r="AG72" s="36"/>
     </row>
     <row r="73" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="19"/>
@@ -5652,116 +5650,116 @@
       <c r="C73" s="21" t="s">
         <v>408</v>
       </c>
-      <c r="D73" s="32" t="s">
+      <c r="D73" s="37" t="s">
         <v>409</v>
       </c>
-      <c r="E73" s="33"/>
-      <c r="F73" s="33"/>
-      <c r="G73" s="33"/>
-      <c r="H73" s="33"/>
-      <c r="I73" s="33"/>
-      <c r="J73" s="33"/>
-      <c r="K73" s="33"/>
-      <c r="L73" s="33"/>
-      <c r="M73" s="33"/>
-      <c r="N73" s="33"/>
-      <c r="O73" s="33"/>
-      <c r="P73" s="33"/>
-      <c r="Q73" s="33"/>
-      <c r="R73" s="33"/>
-      <c r="S73" s="33"/>
-      <c r="T73" s="33"/>
-      <c r="U73" s="33"/>
-      <c r="V73" s="33"/>
-      <c r="W73" s="33"/>
-      <c r="X73" s="33"/>
-      <c r="Y73" s="33"/>
-      <c r="Z73" s="33"/>
-      <c r="AA73" s="33"/>
-      <c r="AB73" s="33"/>
-      <c r="AC73" s="33"/>
-      <c r="AD73" s="33"/>
-      <c r="AE73" s="33"/>
-      <c r="AF73" s="33"/>
-      <c r="AG73" s="34"/>
+      <c r="E73" s="35"/>
+      <c r="F73" s="35"/>
+      <c r="G73" s="35"/>
+      <c r="H73" s="35"/>
+      <c r="I73" s="35"/>
+      <c r="J73" s="35"/>
+      <c r="K73" s="35"/>
+      <c r="L73" s="35"/>
+      <c r="M73" s="35"/>
+      <c r="N73" s="35"/>
+      <c r="O73" s="35"/>
+      <c r="P73" s="35"/>
+      <c r="Q73" s="35"/>
+      <c r="R73" s="35"/>
+      <c r="S73" s="35"/>
+      <c r="T73" s="35"/>
+      <c r="U73" s="35"/>
+      <c r="V73" s="35"/>
+      <c r="W73" s="35"/>
+      <c r="X73" s="35"/>
+      <c r="Y73" s="35"/>
+      <c r="Z73" s="35"/>
+      <c r="AA73" s="35"/>
+      <c r="AB73" s="35"/>
+      <c r="AC73" s="35"/>
+      <c r="AD73" s="35"/>
+      <c r="AE73" s="35"/>
+      <c r="AF73" s="35"/>
+      <c r="AG73" s="36"/>
     </row>
     <row r="74" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="B74" s="36" t="s">
+      <c r="B74" s="38" t="s">
         <v>410</v>
       </c>
-      <c r="C74" s="33"/>
-      <c r="D74" s="33"/>
-      <c r="E74" s="33"/>
-      <c r="F74" s="33"/>
-      <c r="G74" s="33"/>
-      <c r="H74" s="33"/>
-      <c r="I74" s="33"/>
-      <c r="J74" s="33"/>
-      <c r="K74" s="33"/>
-      <c r="L74" s="33"/>
-      <c r="M74" s="33"/>
-      <c r="N74" s="33"/>
-      <c r="O74" s="33"/>
-      <c r="P74" s="33"/>
-      <c r="Q74" s="33"/>
-      <c r="R74" s="33"/>
-      <c r="S74" s="33"/>
-      <c r="T74" s="33"/>
-      <c r="U74" s="33"/>
-      <c r="V74" s="33"/>
-      <c r="W74" s="33"/>
-      <c r="X74" s="33"/>
-      <c r="Y74" s="33"/>
-      <c r="Z74" s="33"/>
-      <c r="AA74" s="33"/>
-      <c r="AB74" s="33"/>
-      <c r="AC74" s="33"/>
-      <c r="AD74" s="33"/>
-      <c r="AE74" s="33"/>
-      <c r="AF74" s="33"/>
-      <c r="AG74" s="34"/>
+      <c r="C74" s="35"/>
+      <c r="D74" s="35"/>
+      <c r="E74" s="35"/>
+      <c r="F74" s="35"/>
+      <c r="G74" s="35"/>
+      <c r="H74" s="35"/>
+      <c r="I74" s="35"/>
+      <c r="J74" s="35"/>
+      <c r="K74" s="35"/>
+      <c r="L74" s="35"/>
+      <c r="M74" s="35"/>
+      <c r="N74" s="35"/>
+      <c r="O74" s="35"/>
+      <c r="P74" s="35"/>
+      <c r="Q74" s="35"/>
+      <c r="R74" s="35"/>
+      <c r="S74" s="35"/>
+      <c r="T74" s="35"/>
+      <c r="U74" s="35"/>
+      <c r="V74" s="35"/>
+      <c r="W74" s="35"/>
+      <c r="X74" s="35"/>
+      <c r="Y74" s="35"/>
+      <c r="Z74" s="35"/>
+      <c r="AA74" s="35"/>
+      <c r="AB74" s="35"/>
+      <c r="AC74" s="35"/>
+      <c r="AD74" s="35"/>
+      <c r="AE74" s="35"/>
+      <c r="AF74" s="35"/>
+      <c r="AG74" s="36"/>
     </row>
     <row r="75" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="B75" s="32" t="s">
+      <c r="B75" s="37" t="s">
         <v>411</v>
       </c>
-      <c r="C75" s="33"/>
-      <c r="D75" s="33"/>
-      <c r="E75" s="33"/>
-      <c r="F75" s="33"/>
-      <c r="G75" s="33"/>
-      <c r="H75" s="33"/>
-      <c r="I75" s="33"/>
-      <c r="J75" s="33"/>
-      <c r="K75" s="33"/>
-      <c r="L75" s="33"/>
-      <c r="M75" s="33"/>
-      <c r="N75" s="33"/>
-      <c r="O75" s="33"/>
-      <c r="P75" s="33"/>
-      <c r="Q75" s="33"/>
-      <c r="R75" s="33"/>
-      <c r="S75" s="33"/>
-      <c r="T75" s="33"/>
-      <c r="U75" s="33"/>
-      <c r="V75" s="33"/>
-      <c r="W75" s="33"/>
-      <c r="X75" s="33"/>
-      <c r="Y75" s="33"/>
-      <c r="Z75" s="33"/>
-      <c r="AA75" s="33"/>
-      <c r="AB75" s="33"/>
-      <c r="AC75" s="33"/>
-      <c r="AD75" s="33"/>
-      <c r="AE75" s="33"/>
-      <c r="AF75" s="33"/>
-      <c r="AG75" s="34"/>
+      <c r="C75" s="35"/>
+      <c r="D75" s="35"/>
+      <c r="E75" s="35"/>
+      <c r="F75" s="35"/>
+      <c r="G75" s="35"/>
+      <c r="H75" s="35"/>
+      <c r="I75" s="35"/>
+      <c r="J75" s="35"/>
+      <c r="K75" s="35"/>
+      <c r="L75" s="35"/>
+      <c r="M75" s="35"/>
+      <c r="N75" s="35"/>
+      <c r="O75" s="35"/>
+      <c r="P75" s="35"/>
+      <c r="Q75" s="35"/>
+      <c r="R75" s="35"/>
+      <c r="S75" s="35"/>
+      <c r="T75" s="35"/>
+      <c r="U75" s="35"/>
+      <c r="V75" s="35"/>
+      <c r="W75" s="35"/>
+      <c r="X75" s="35"/>
+      <c r="Y75" s="35"/>
+      <c r="Z75" s="35"/>
+      <c r="AA75" s="35"/>
+      <c r="AB75" s="35"/>
+      <c r="AC75" s="35"/>
+      <c r="AD75" s="35"/>
+      <c r="AE75" s="35"/>
+      <c r="AF75" s="35"/>
+      <c r="AG75" s="36"/>
     </row>
     <row r="76" spans="1:33" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="23" t="s">
@@ -5947,79 +5945,79 @@
       <c r="A92" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B92" s="36" t="s">
+      <c r="B92" s="38" t="s">
         <v>423</v>
       </c>
-      <c r="C92" s="33"/>
-      <c r="D92" s="33"/>
-      <c r="E92" s="33"/>
-      <c r="F92" s="33"/>
-      <c r="G92" s="33"/>
-      <c r="H92" s="33"/>
-      <c r="I92" s="33"/>
-      <c r="J92" s="33"/>
-      <c r="K92" s="33"/>
-      <c r="L92" s="33"/>
-      <c r="M92" s="33"/>
-      <c r="N92" s="33"/>
-      <c r="O92" s="33"/>
-      <c r="P92" s="33"/>
-      <c r="Q92" s="33"/>
-      <c r="R92" s="33"/>
-      <c r="S92" s="33"/>
-      <c r="T92" s="33"/>
-      <c r="U92" s="33"/>
-      <c r="V92" s="33"/>
-      <c r="W92" s="33"/>
-      <c r="X92" s="33"/>
-      <c r="Y92" s="33"/>
-      <c r="Z92" s="33"/>
-      <c r="AA92" s="33"/>
-      <c r="AB92" s="33"/>
-      <c r="AC92" s="33"/>
-      <c r="AD92" s="33"/>
-      <c r="AE92" s="33"/>
-      <c r="AF92" s="33"/>
-      <c r="AG92" s="34"/>
+      <c r="C92" s="35"/>
+      <c r="D92" s="35"/>
+      <c r="E92" s="35"/>
+      <c r="F92" s="35"/>
+      <c r="G92" s="35"/>
+      <c r="H92" s="35"/>
+      <c r="I92" s="35"/>
+      <c r="J92" s="35"/>
+      <c r="K92" s="35"/>
+      <c r="L92" s="35"/>
+      <c r="M92" s="35"/>
+      <c r="N92" s="35"/>
+      <c r="O92" s="35"/>
+      <c r="P92" s="35"/>
+      <c r="Q92" s="35"/>
+      <c r="R92" s="35"/>
+      <c r="S92" s="35"/>
+      <c r="T92" s="35"/>
+      <c r="U92" s="35"/>
+      <c r="V92" s="35"/>
+      <c r="W92" s="35"/>
+      <c r="X92" s="35"/>
+      <c r="Y92" s="35"/>
+      <c r="Z92" s="35"/>
+      <c r="AA92" s="35"/>
+      <c r="AB92" s="35"/>
+      <c r="AC92" s="35"/>
+      <c r="AD92" s="35"/>
+      <c r="AE92" s="35"/>
+      <c r="AF92" s="35"/>
+      <c r="AG92" s="36"/>
     </row>
     <row r="93" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="B93" s="32" t="s">
+      <c r="B93" s="37" t="s">
         <v>424</v>
       </c>
-      <c r="C93" s="33"/>
-      <c r="D93" s="33"/>
-      <c r="E93" s="33"/>
-      <c r="F93" s="33"/>
-      <c r="G93" s="33"/>
-      <c r="H93" s="33"/>
-      <c r="I93" s="33"/>
-      <c r="J93" s="33"/>
-      <c r="K93" s="33"/>
-      <c r="L93" s="33"/>
-      <c r="M93" s="33"/>
-      <c r="N93" s="33"/>
-      <c r="O93" s="33"/>
-      <c r="P93" s="33"/>
-      <c r="Q93" s="33"/>
-      <c r="R93" s="33"/>
-      <c r="S93" s="33"/>
-      <c r="T93" s="33"/>
-      <c r="U93" s="33"/>
-      <c r="V93" s="33"/>
-      <c r="W93" s="33"/>
-      <c r="X93" s="33"/>
-      <c r="Y93" s="33"/>
-      <c r="Z93" s="33"/>
-      <c r="AA93" s="33"/>
-      <c r="AB93" s="33"/>
-      <c r="AC93" s="33"/>
-      <c r="AD93" s="33"/>
-      <c r="AE93" s="33"/>
-      <c r="AF93" s="33"/>
-      <c r="AG93" s="34"/>
+      <c r="C93" s="35"/>
+      <c r="D93" s="35"/>
+      <c r="E93" s="35"/>
+      <c r="F93" s="35"/>
+      <c r="G93" s="35"/>
+      <c r="H93" s="35"/>
+      <c r="I93" s="35"/>
+      <c r="J93" s="35"/>
+      <c r="K93" s="35"/>
+      <c r="L93" s="35"/>
+      <c r="M93" s="35"/>
+      <c r="N93" s="35"/>
+      <c r="O93" s="35"/>
+      <c r="P93" s="35"/>
+      <c r="Q93" s="35"/>
+      <c r="R93" s="35"/>
+      <c r="S93" s="35"/>
+      <c r="T93" s="35"/>
+      <c r="U93" s="35"/>
+      <c r="V93" s="35"/>
+      <c r="W93" s="35"/>
+      <c r="X93" s="35"/>
+      <c r="Y93" s="35"/>
+      <c r="Z93" s="35"/>
+      <c r="AA93" s="35"/>
+      <c r="AB93" s="35"/>
+      <c r="AC93" s="35"/>
+      <c r="AD93" s="35"/>
+      <c r="AE93" s="35"/>
+      <c r="AF93" s="35"/>
+      <c r="AG93" s="36"/>
     </row>
     <row r="94" spans="1:33" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="19" t="s">
@@ -6031,38 +6029,38 @@
       <c r="C94" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="D94" s="35" t="s">
+      <c r="D94" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="E94" s="33"/>
-      <c r="F94" s="33"/>
-      <c r="G94" s="33"/>
-      <c r="H94" s="33"/>
-      <c r="I94" s="33"/>
-      <c r="J94" s="33"/>
-      <c r="K94" s="33"/>
-      <c r="L94" s="33"/>
-      <c r="M94" s="33"/>
-      <c r="N94" s="33"/>
-      <c r="O94" s="33"/>
-      <c r="P94" s="33"/>
-      <c r="Q94" s="33"/>
-      <c r="R94" s="33"/>
-      <c r="S94" s="33"/>
-      <c r="T94" s="33"/>
-      <c r="U94" s="33"/>
-      <c r="V94" s="33"/>
-      <c r="W94" s="33"/>
-      <c r="X94" s="33"/>
-      <c r="Y94" s="33"/>
-      <c r="Z94" s="33"/>
-      <c r="AA94" s="33"/>
-      <c r="AB94" s="33"/>
-      <c r="AC94" s="33"/>
-      <c r="AD94" s="33"/>
-      <c r="AE94" s="33"/>
-      <c r="AF94" s="33"/>
-      <c r="AG94" s="34"/>
+      <c r="E94" s="35"/>
+      <c r="F94" s="35"/>
+      <c r="G94" s="35"/>
+      <c r="H94" s="35"/>
+      <c r="I94" s="35"/>
+      <c r="J94" s="35"/>
+      <c r="K94" s="35"/>
+      <c r="L94" s="35"/>
+      <c r="M94" s="35"/>
+      <c r="N94" s="35"/>
+      <c r="O94" s="35"/>
+      <c r="P94" s="35"/>
+      <c r="Q94" s="35"/>
+      <c r="R94" s="35"/>
+      <c r="S94" s="35"/>
+      <c r="T94" s="35"/>
+      <c r="U94" s="35"/>
+      <c r="V94" s="35"/>
+      <c r="W94" s="35"/>
+      <c r="X94" s="35"/>
+      <c r="Y94" s="35"/>
+      <c r="Z94" s="35"/>
+      <c r="AA94" s="35"/>
+      <c r="AB94" s="35"/>
+      <c r="AC94" s="35"/>
+      <c r="AD94" s="35"/>
+      <c r="AE94" s="35"/>
+      <c r="AF94" s="35"/>
+      <c r="AG94" s="36"/>
     </row>
     <row r="95" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="19"/>
@@ -6072,116 +6070,116 @@
       <c r="C95" s="21" t="s">
         <v>425</v>
       </c>
-      <c r="D95" s="32" t="s">
+      <c r="D95" s="37" t="s">
         <v>426</v>
       </c>
-      <c r="E95" s="33"/>
-      <c r="F95" s="33"/>
-      <c r="G95" s="33"/>
-      <c r="H95" s="33"/>
-      <c r="I95" s="33"/>
-      <c r="J95" s="33"/>
-      <c r="K95" s="33"/>
-      <c r="L95" s="33"/>
-      <c r="M95" s="33"/>
-      <c r="N95" s="33"/>
-      <c r="O95" s="33"/>
-      <c r="P95" s="33"/>
-      <c r="Q95" s="33"/>
-      <c r="R95" s="33"/>
-      <c r="S95" s="33"/>
-      <c r="T95" s="33"/>
-      <c r="U95" s="33"/>
-      <c r="V95" s="33"/>
-      <c r="W95" s="33"/>
-      <c r="X95" s="33"/>
-      <c r="Y95" s="33"/>
-      <c r="Z95" s="33"/>
-      <c r="AA95" s="33"/>
-      <c r="AB95" s="33"/>
-      <c r="AC95" s="33"/>
-      <c r="AD95" s="33"/>
-      <c r="AE95" s="33"/>
-      <c r="AF95" s="33"/>
-      <c r="AG95" s="34"/>
+      <c r="E95" s="35"/>
+      <c r="F95" s="35"/>
+      <c r="G95" s="35"/>
+      <c r="H95" s="35"/>
+      <c r="I95" s="35"/>
+      <c r="J95" s="35"/>
+      <c r="K95" s="35"/>
+      <c r="L95" s="35"/>
+      <c r="M95" s="35"/>
+      <c r="N95" s="35"/>
+      <c r="O95" s="35"/>
+      <c r="P95" s="35"/>
+      <c r="Q95" s="35"/>
+      <c r="R95" s="35"/>
+      <c r="S95" s="35"/>
+      <c r="T95" s="35"/>
+      <c r="U95" s="35"/>
+      <c r="V95" s="35"/>
+      <c r="W95" s="35"/>
+      <c r="X95" s="35"/>
+      <c r="Y95" s="35"/>
+      <c r="Z95" s="35"/>
+      <c r="AA95" s="35"/>
+      <c r="AB95" s="35"/>
+      <c r="AC95" s="35"/>
+      <c r="AD95" s="35"/>
+      <c r="AE95" s="35"/>
+      <c r="AF95" s="35"/>
+      <c r="AG95" s="36"/>
     </row>
     <row r="96" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="B96" s="36" t="s">
+      <c r="B96" s="38" t="s">
         <v>427</v>
       </c>
-      <c r="C96" s="33"/>
-      <c r="D96" s="33"/>
-      <c r="E96" s="33"/>
-      <c r="F96" s="33"/>
-      <c r="G96" s="33"/>
-      <c r="H96" s="33"/>
-      <c r="I96" s="33"/>
-      <c r="J96" s="33"/>
-      <c r="K96" s="33"/>
-      <c r="L96" s="33"/>
-      <c r="M96" s="33"/>
-      <c r="N96" s="33"/>
-      <c r="O96" s="33"/>
-      <c r="P96" s="33"/>
-      <c r="Q96" s="33"/>
-      <c r="R96" s="33"/>
-      <c r="S96" s="33"/>
-      <c r="T96" s="33"/>
-      <c r="U96" s="33"/>
-      <c r="V96" s="33"/>
-      <c r="W96" s="33"/>
-      <c r="X96" s="33"/>
-      <c r="Y96" s="33"/>
-      <c r="Z96" s="33"/>
-      <c r="AA96" s="33"/>
-      <c r="AB96" s="33"/>
-      <c r="AC96" s="33"/>
-      <c r="AD96" s="33"/>
-      <c r="AE96" s="33"/>
-      <c r="AF96" s="33"/>
-      <c r="AG96" s="34"/>
+      <c r="C96" s="35"/>
+      <c r="D96" s="35"/>
+      <c r="E96" s="35"/>
+      <c r="F96" s="35"/>
+      <c r="G96" s="35"/>
+      <c r="H96" s="35"/>
+      <c r="I96" s="35"/>
+      <c r="J96" s="35"/>
+      <c r="K96" s="35"/>
+      <c r="L96" s="35"/>
+      <c r="M96" s="35"/>
+      <c r="N96" s="35"/>
+      <c r="O96" s="35"/>
+      <c r="P96" s="35"/>
+      <c r="Q96" s="35"/>
+      <c r="R96" s="35"/>
+      <c r="S96" s="35"/>
+      <c r="T96" s="35"/>
+      <c r="U96" s="35"/>
+      <c r="V96" s="35"/>
+      <c r="W96" s="35"/>
+      <c r="X96" s="35"/>
+      <c r="Y96" s="35"/>
+      <c r="Z96" s="35"/>
+      <c r="AA96" s="35"/>
+      <c r="AB96" s="35"/>
+      <c r="AC96" s="35"/>
+      <c r="AD96" s="35"/>
+      <c r="AE96" s="35"/>
+      <c r="AF96" s="35"/>
+      <c r="AG96" s="36"/>
     </row>
     <row r="97" spans="1:33" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="B97" s="32" t="s">
+      <c r="B97" s="37" t="s">
         <v>428</v>
       </c>
-      <c r="C97" s="33"/>
-      <c r="D97" s="33"/>
-      <c r="E97" s="33"/>
-      <c r="F97" s="33"/>
-      <c r="G97" s="33"/>
-      <c r="H97" s="33"/>
-      <c r="I97" s="33"/>
-      <c r="J97" s="33"/>
-      <c r="K97" s="33"/>
-      <c r="L97" s="33"/>
-      <c r="M97" s="33"/>
-      <c r="N97" s="33"/>
-      <c r="O97" s="33"/>
-      <c r="P97" s="33"/>
-      <c r="Q97" s="33"/>
-      <c r="R97" s="33"/>
-      <c r="S97" s="33"/>
-      <c r="T97" s="33"/>
-      <c r="U97" s="33"/>
-      <c r="V97" s="33"/>
-      <c r="W97" s="33"/>
-      <c r="X97" s="33"/>
-      <c r="Y97" s="33"/>
-      <c r="Z97" s="33"/>
-      <c r="AA97" s="33"/>
-      <c r="AB97" s="33"/>
-      <c r="AC97" s="33"/>
-      <c r="AD97" s="33"/>
-      <c r="AE97" s="33"/>
-      <c r="AF97" s="33"/>
-      <c r="AG97" s="34"/>
+      <c r="C97" s="35"/>
+      <c r="D97" s="35"/>
+      <c r="E97" s="35"/>
+      <c r="F97" s="35"/>
+      <c r="G97" s="35"/>
+      <c r="H97" s="35"/>
+      <c r="I97" s="35"/>
+      <c r="J97" s="35"/>
+      <c r="K97" s="35"/>
+      <c r="L97" s="35"/>
+      <c r="M97" s="35"/>
+      <c r="N97" s="35"/>
+      <c r="O97" s="35"/>
+      <c r="P97" s="35"/>
+      <c r="Q97" s="35"/>
+      <c r="R97" s="35"/>
+      <c r="S97" s="35"/>
+      <c r="T97" s="35"/>
+      <c r="U97" s="35"/>
+      <c r="V97" s="35"/>
+      <c r="W97" s="35"/>
+      <c r="X97" s="35"/>
+      <c r="Y97" s="35"/>
+      <c r="Z97" s="35"/>
+      <c r="AA97" s="35"/>
+      <c r="AB97" s="35"/>
+      <c r="AC97" s="35"/>
+      <c r="AD97" s="35"/>
+      <c r="AE97" s="35"/>
+      <c r="AF97" s="35"/>
+      <c r="AG97" s="36"/>
     </row>
     <row r="98" spans="1:33" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="23" t="s">
@@ -6392,14 +6390,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A1:U1"/>
-    <mergeCell ref="D94:AG94"/>
-    <mergeCell ref="D50:AG50"/>
-    <mergeCell ref="B9:AG9"/>
-    <mergeCell ref="B49:AG49"/>
-    <mergeCell ref="B74:AG74"/>
-    <mergeCell ref="B92:AG92"/>
-    <mergeCell ref="B30:AG30"/>
     <mergeCell ref="D95:AG95"/>
     <mergeCell ref="B97:AG97"/>
     <mergeCell ref="A2:U2"/>
@@ -6416,6 +6406,14 @@
     <mergeCell ref="D28:AG28"/>
     <mergeCell ref="B8:AG8"/>
     <mergeCell ref="D29:AG29"/>
+    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="D94:AG94"/>
+    <mergeCell ref="D50:AG50"/>
+    <mergeCell ref="B9:AG9"/>
+    <mergeCell ref="B49:AG49"/>
+    <mergeCell ref="B74:AG74"/>
+    <mergeCell ref="B92:AG92"/>
+    <mergeCell ref="B30:AG30"/>
     <mergeCell ref="B5:AG5"/>
     <mergeCell ref="D6:AG6"/>
     <mergeCell ref="B4:AG4"/>
@@ -6444,24 +6442,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="4" spans="1:6" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
@@ -6610,24 +6608,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="39" t="s">
         <v>438</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="4" spans="1:6" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">

</xml_diff>